<commit_message>
update dashboard and csv's
</commit_message>
<xml_diff>
--- a/bucket_1_connector_features.xlsx
+++ b/bucket_1_connector_features.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G197"/>
+  <dimension ref="A1:G182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -654,7 +654,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2758,27 +2758,27 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>adyen</t>
+          <t>santander</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Push Notification Flow</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Handle bank-initiated push notification to trigger a new mandate charge cycle (e.g. PIX Automático)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /payments (internal mandate push notification)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2791,27 +2791,27 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>barclaycard</t>
+          <t>santander</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>QR Code Generation Flow</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Generate a scannable QR code for the payment (e.g. PIX, WeChat Pay, GrabPay)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /payments (internal QR code generation)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2824,27 +2824,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>blackhawknetwork</t>
+          <t>aci</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -2857,55 +2857,59 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>cybersource</t>
+          <t>adyen</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-04-21 01:36:11</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>gocardless</t>
+          <t>affirm</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2923,64 +2927,60 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>nexixpay</t>
+          <t>airwallex</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2026-02-05 22:14:48.025</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>nmi</t>
+          <t>amazonpay</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -2993,27 +2993,27 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>nordea</t>
+          <t>archipel</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3026,97 +3026,97 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>nuvei</t>
+          <t>authipay</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>2026-02-04 07:43:53.078</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>payme</t>
+          <t>authorizedotnet</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-04-20 19:45:30</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>paypal</t>
+          <t>bambora</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3129,27 +3129,27 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>paysafe</t>
+          <t>bamboraapac</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3162,64 +3162,60 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>redsys</t>
+          <t>bankofamerica</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>2026-02-05 16:51:52.490</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>shift4</t>
+          <t>barclaycard</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3232,27 +3228,27 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>trustpay</t>
+          <t>billwerk</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3265,27 +3261,27 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>xendit</t>
+          <t>bitpay</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Preprocessing Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Connector-specific setup step before authorization (e.g. session creation, device fingerprinting, BNPL eligibility check)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>POST /payments (internal preprocessing before auth)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3298,27 +3294,27 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>santander</t>
+          <t>bluesnap</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Push Notification Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Handle bank-initiated push notification to trigger a new mandate charge cycle (e.g. PIX Automático)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>POST /payments (internal mandate push notification)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3331,22 +3327,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>santander</t>
+          <t>boku</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>QR Code Generation Flow</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Generate a scannable QR code for the payment (e.g. PIX, WeChat Pay, GrabPay)</t>
+          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>POST /payments (internal QR code generation)</t>
+          <t>POST /refunds</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3364,7 +3360,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>aci</t>
+          <t>braintree</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3397,7 +3393,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>adyen</t>
+          <t>breadpay</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3417,24 +3413,20 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>2026-04-21 01:36:11</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>affirm</t>
+          <t>celero</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3454,7 +3446,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3467,7 +3459,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>airwallex</t>
+          <t>checkout</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3500,7 +3492,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>amazonpay</t>
+          <t>coingate</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3533,7 +3525,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>archipel</t>
+          <t>cybersource</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -3558,15 +3550,19 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2026-04-20 15:16:44</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>authipay</t>
+          <t>datatrans</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3599,7 +3595,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>authorizedotnet</t>
+          <t>deutschebank</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3624,19 +3620,15 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>2026-04-20 19:45:30</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>bambora</t>
+          <t>digitalvirgo</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3656,7 +3648,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -3669,7 +3661,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>bamboraapac</t>
+          <t>dlocal</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3702,7 +3694,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>bankofamerica</t>
+          <t>dwolla</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3722,7 +3714,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -3735,7 +3727,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>barclaycard</t>
+          <t>elavon</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3768,7 +3760,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>billwerk</t>
+          <t>facilitapay</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3788,7 +3780,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -3801,7 +3793,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>bitpay</t>
+          <t>finix</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3821,20 +3813,24 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2026-04-18 19:43:27</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>bluesnap</t>
+          <t>fiserv</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3867,7 +3863,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>boku</t>
+          <t>fiservcommercehub</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3900,7 +3896,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>braintree</t>
+          <t>fiservemea</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3933,7 +3929,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>breadpay</t>
+          <t>fiuu</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3953,20 +3949,24 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:10:27</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>celero</t>
+          <t>forte</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3999,7 +3999,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>checkout</t>
+          <t>getnet</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -4032,7 +4032,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>coingate</t>
+          <t>gigadat</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -4065,7 +4065,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>cybersource</t>
+          <t>globalpay</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -4090,19 +4090,15 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>2026-04-20 15:16:44</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>datatrans</t>
+          <t>globepay</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -4122,7 +4118,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -4135,7 +4131,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>deutschebank</t>
+          <t>gocardless</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -4155,7 +4151,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -4168,7 +4164,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>digitalvirgo</t>
+          <t>helcim</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -4201,7 +4197,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>dlocal</t>
+          <t>hipay</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -4234,7 +4230,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>dwolla</t>
+          <t>hyperpg</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -4267,7 +4263,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>elavon</t>
+          <t>iatapay</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -4300,7 +4296,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>facilitapay</t>
+          <t>imerchantsolutions</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -4320,7 +4316,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -4333,7 +4329,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>finix</t>
+          <t>inespay</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -4353,24 +4349,20 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>2026-04-18 19:43:27</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>fiserv</t>
+          <t>itaubank</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -4390,7 +4382,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -4403,7 +4395,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>fiservcommercehub</t>
+          <t>jpmorgan</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -4423,7 +4415,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -4436,7 +4428,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>fiservemea</t>
+          <t>klarna</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -4456,7 +4448,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -4469,7 +4461,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>fiuu</t>
+          <t>loonio</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -4489,24 +4481,20 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>2026-04-19 09:10:27</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>forte</t>
+          <t>mollie</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -4539,7 +4527,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>getnet</t>
+          <t>moneris</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -4572,7 +4560,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>gigadat</t>
+          <t>multisafepay</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -4592,7 +4580,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -4605,7 +4593,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>globalpay</t>
+          <t>nexinets</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -4638,7 +4626,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>globepay</t>
+          <t>nexixpay</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -4658,20 +4646,24 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-03-02 07:48:10</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>gocardless</t>
+          <t>nmi</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -4691,20 +4683,24 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-04-20 17:12:33</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>helcim</t>
+          <t>noon</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -4724,20 +4720,24 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>2026-04-21 00:25:18</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>hipay</t>
+          <t>novalnet</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -4762,15 +4762,19 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-04-20 21:01:29</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>hyperpg</t>
+          <t>nuvei</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -4790,7 +4794,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -4803,7 +4807,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>iatapay</t>
+          <t>paybox</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -4836,7 +4840,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>inespay</t>
+          <t>payeezy</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -4869,7 +4873,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>itaubank</t>
+          <t>payjustnow</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -4889,7 +4893,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -4902,7 +4906,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>jpmorgan</t>
+          <t>payjustnowinstore</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -4922,7 +4926,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -4935,7 +4939,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>klarna</t>
+          <t>payload</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -4955,7 +4959,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -4968,7 +4972,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>loonio</t>
+          <t>payme</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -4988,7 +4992,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -5001,7 +5005,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>mollie</t>
+          <t>paypal</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -5026,15 +5030,19 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G138" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2026-04-20 12:20:22</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>moneris</t>
+          <t>paysafe</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -5067,7 +5075,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>multisafepay</t>
+          <t>paystack</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5087,7 +5095,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -5100,7 +5108,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>nexinets</t>
+          <t>payu</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -5133,7 +5141,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>nexixpay</t>
+          <t>peachpayments</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -5163,14 +5171,14 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-03-02 07:48:10</t>
+          <t>2026-04-08 10:11:19</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>nmi</t>
+          <t>placetopay</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -5190,24 +5198,20 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>2026-04-20 17:12:33</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>noon</t>
+          <t>powertranz</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -5232,19 +5236,15 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>2026-04-21 00:25:18</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>novalnet</t>
+          <t>prophetpay</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -5264,24 +5264,20 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>2026-04-20 21:01:29</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>nuvei</t>
+          <t>rapyd</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -5301,7 +5297,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -5314,7 +5310,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>paybox</t>
+          <t>razorpay</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -5334,7 +5330,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -5347,7 +5343,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>payeezy</t>
+          <t>redsys</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -5367,7 +5363,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -5380,7 +5376,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>payjustnow</t>
+          <t>revolv3</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -5413,7 +5409,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>payjustnowinstore</t>
+          <t>santander</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -5446,7 +5442,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>payload</t>
+          <t>shift4</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -5479,7 +5475,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>payme</t>
+          <t>silverflow</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -5499,7 +5495,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -5512,7 +5508,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>paypal</t>
+          <t>square</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -5537,19 +5533,15 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>2026-04-20 12:20:22</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>paysafe</t>
+          <t>stax</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -5582,7 +5574,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>paystack</t>
+          <t>stripe</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -5602,20 +5594,24 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G155" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2026-04-21 01:32:04</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>payu</t>
+          <t>tesouro</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -5648,7 +5644,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>peachpayments</t>
+          <t>truelayer</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -5668,24 +5664,20 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>2026-04-08 10:11:19</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>placetopay</t>
+          <t>trustly</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -5718,7 +5710,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>powertranz</t>
+          <t>trustpay</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -5743,15 +5735,19 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G159" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:14:11</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>prophetpay</t>
+          <t>trustpayments</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -5771,7 +5767,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -5784,7 +5780,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>rapyd</t>
+          <t>tsys</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -5804,7 +5800,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -5817,7 +5813,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>razorpay</t>
+          <t>volt</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -5837,7 +5833,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -5850,7 +5846,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>redsys</t>
+          <t>wellsfargo</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -5883,7 +5879,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>revolv3</t>
+          <t>worldline</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -5916,7 +5912,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>santander</t>
+          <t>worldpay</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -5936,20 +5932,24 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G165" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>2026-04-06 05:02:32</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>shift4</t>
+          <t>worldpaymodular</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -5982,7 +5982,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>silverflow</t>
+          <t>worldpayvantiv</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -6015,7 +6015,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>square</t>
+          <t>worldpayxml</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -6040,15 +6040,19 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>2026-03-23 06:31:48</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>stax</t>
+          <t>xendit</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -6081,7 +6085,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>stripe</t>
+          <t>zen</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -6101,24 +6105,20 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>2026-04-21 01:32:04</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>tesouro</t>
+          <t>zift</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -6151,27 +6151,27 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>truelayer</t>
+          <t>xendit</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Settlement Split Call</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Split settlement amounts across sub-merchants or accounts after authorization</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /payments (internal post-auth settlement split)</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -6184,32 +6184,32 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>trustly</t>
+          <t>adyen</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Split Payments</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Split a single payment across multiple accounts or sub-merchant recipients</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /payments (split_payments in body)</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="G173" t="inlineStr"/>
@@ -6217,22 +6217,22 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>trustpay</t>
+          <t>stripe</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Split Payments</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Split a single payment across multiple accounts or sub-merchant recipients</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /payments (split_payments in body)</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -6242,44 +6242,40 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>2026-04-20 10:14:11</t>
-        </is>
-      </c>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>trustpayments</t>
+          <t>xendit</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Split Payments</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Split a single payment across multiple accounts or sub-merchant recipients</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /payments (split_payments in body)</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="G175" t="inlineStr"/>
@@ -6287,93 +6283,101 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>tsys</t>
+          <t>adyen</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Split Refunds</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Refund a split payment proportionally across the original split recipients</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /refunds (split_refunds in body)</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G176" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>2026-04-21 01:36:11</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>volt</t>
+          <t>stripe</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Split Refunds</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Refund a split payment proportionally across the original split recipients</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /refunds (split_refunds in body)</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>not_covered</t>
+          <t>covered</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G177" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>2026-04-20 17:12:49</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>wellsfargo</t>
+          <t>xendit</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Split Refunds</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Refund a split payment proportionally across the original split recipients</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /refunds (split_refunds in body)</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -6386,27 +6390,27 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>worldline</t>
+          <t>barclaycard</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Step Up Authentication</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Trigger a 3DS step-up challenge when a prior frictionless flow is deemed insufficient by the issuer</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /payments (internal 3DS2 step-up redirect)</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -6419,64 +6423,60 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>worldpay</t>
+          <t>cybersource</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Step Up Authentication</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Trigger a 3DS step-up challenge when a prior frictionless flow is deemed insufficient by the issuer</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /payments (internal 3DS2 step-up redirect)</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>2026-04-06 05:02:32</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>worldpaymodular</t>
+          <t>celero</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Surcharge</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Add a connector-forwarded surcharge fee on top of the payment amount</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /payments (surcharge_details in body)</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>no_cypress_config</t>
+          <t>not_covered</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -6489,27 +6489,27 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>worldpayvantiv</t>
+          <t>digitalvirgo</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Surcharge</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
+          <t>Add a connector-forwarded surcharge fee on top of the payment amount</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>POST /refunds</t>
+          <t>POST /payments (surcharge_details in body)</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>covered</t>
+          <t>no_cypress_config</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -6518,513 +6518,6 @@
         </is>
       </c>
       <c r="G182" t="inlineStr"/>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>worldpayxml</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>Refund</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>POST /refunds</t>
-        </is>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>covered</t>
-        </is>
-      </c>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>2026-03-23 06:31:48</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>xendit</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>Refund</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
-        </is>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>POST /refunds</t>
-        </is>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>covered</t>
-        </is>
-      </c>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr"/>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>zen</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>Refund</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>POST /refunds</t>
-        </is>
-      </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>no_cypress_config</t>
-        </is>
-      </c>
-      <c r="F185" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G185" t="inlineStr"/>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>zift</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>Refund</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>Connector supports refund of a completed payment (at least one PM/PMT combination)</t>
-        </is>
-      </c>
-      <c r="D186" t="inlineStr">
-        <is>
-          <t>POST /refunds</t>
-        </is>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>covered</t>
-        </is>
-      </c>
-      <c r="F186" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G186" t="inlineStr"/>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>xendit</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>Settlement Split Call</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>Split settlement amounts across sub-merchants or accounts after authorization</t>
-        </is>
-      </c>
-      <c r="D187" t="inlineStr">
-        <is>
-          <t>POST /payments (internal post-auth settlement split)</t>
-        </is>
-      </c>
-      <c r="E187" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F187" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G187" t="inlineStr"/>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>adyen</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>Split Payments</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>Split a single payment across multiple accounts or sub-merchant recipients</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>POST /payments (split_payments in body)</t>
-        </is>
-      </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F188" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="G188" t="inlineStr"/>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>stripe</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>Split Payments</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>Split a single payment across multiple accounts or sub-merchant recipients</t>
-        </is>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>POST /payments (split_payments in body)</t>
-        </is>
-      </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F189" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="G189" t="inlineStr"/>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>xendit</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>Split Payments</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>Split a single payment across multiple accounts or sub-merchant recipients</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>POST /payments (split_payments in body)</t>
-        </is>
-      </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F190" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="G190" t="inlineStr"/>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>adyen</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>Split Refunds</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>Refund a split payment proportionally across the original split recipients</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>POST /refunds (split_refunds in body)</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F191" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>2026-04-21 01:36:11</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>stripe</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>Split Refunds</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>Refund a split payment proportionally across the original split recipients</t>
-        </is>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>POST /refunds (split_refunds in body)</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>2026-04-20 17:12:49</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>xendit</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>Split Refunds</t>
-        </is>
-      </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>Refund a split payment proportionally across the original split recipients</t>
-        </is>
-      </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>POST /refunds (split_refunds in body)</t>
-        </is>
-      </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F193" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G193" t="inlineStr"/>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>barclaycard</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>Step Up Authentication</t>
-        </is>
-      </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>Trigger a 3DS step-up challenge when a prior frictionless flow is deemed insufficient by the issuer</t>
-        </is>
-      </c>
-      <c r="D194" t="inlineStr">
-        <is>
-          <t>POST /payments (internal 3DS2 step-up redirect)</t>
-        </is>
-      </c>
-      <c r="E194" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F194" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G194" t="inlineStr"/>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>cybersource</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>Step Up Authentication</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>Trigger a 3DS step-up challenge when a prior frictionless flow is deemed insufficient by the issuer</t>
-        </is>
-      </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>POST /payments (internal 3DS2 step-up redirect)</t>
-        </is>
-      </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F195" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G195" t="inlineStr"/>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>celero</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>Surcharge</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>Add a connector-forwarded surcharge fee on top of the payment amount</t>
-        </is>
-      </c>
-      <c r="D196" t="inlineStr">
-        <is>
-          <t>POST /payments (surcharge_details in body)</t>
-        </is>
-      </c>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>not_covered</t>
-        </is>
-      </c>
-      <c r="F196" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G196" t="inlineStr"/>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>digitalvirgo</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>Surcharge</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>Add a connector-forwarded surcharge fee on top of the payment amount</t>
-        </is>
-      </c>
-      <c r="D197" t="inlineStr">
-        <is>
-          <t>POST /payments (surcharge_details in body)</t>
-        </is>
-      </c>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>no_cypress_config</t>
-        </is>
-      </c>
-      <c r="F197" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G197" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>